<commit_message>
Deployed 4809e8a with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/Buch Camille Chronicles/Zeitlinie_Soulbound.xlsx
+++ b/Buch Camille Chronicles/Zeitlinie_Soulbound.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian Dauner\Documents\GitHub\pnpWiki\docs\Buch Camille Chronicles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64BC7962-652E-46A3-B1EC-448B4ACA7C21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC6A1844-A1F3-44B1-B0DD-6EFDE1EBED29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5205" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Monat</t>
   </si>
@@ -48,24 +48,43 @@
     <t>Death of Bureaucratess Nalil 
 Camill going to Asarat's Peak
 Camill checks into the bar 'Ubir Ubar’</t>
-  </si>
-  <si>
-    <t>Camill fights her first opponent in the Arena</t>
   </si>
   <si>
     <t>Camill gets thrown from the bar
 Camill attends The Receiving and has a vision from the Immortal Oracle
 Camill gets thrown out of a mercenaries post
 Camill decides to collect moeny for winning in the Arena.</t>
+  </si>
+  <si>
+    <t>Camill fights her first opponent in the Arena
+Camill has to fight her second fight against Natrair
+Riots break out in the Arena
+Camill flees accidently to the Temple of Sun and Moon</t>
+  </si>
+  <si>
+    <t>Jahr a.C.</t>
+  </si>
+  <si>
+    <t>Shkaratve</t>
+  </si>
+  <si>
+    <t>Camill's birthday</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -92,11 +111,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -377,59 +397,80 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>3739</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="2">
+        <v>3761</v>
+      </c>
+      <c r="B5" t="s">
         <v>4</v>
       </c>
-      <c r="B2">
+      <c r="C5">
         <v>52</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="144" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+    <row r="6" spans="1:5" ht="144" x14ac:dyDescent="0.3">
+      <c r="A6" s="2"/>
+      <c r="B6" t="s">
         <v>5</v>
       </c>
-      <c r="B3">
+      <c r="C6">
         <v>1</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D6" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B4">
-        <v>2</v>
-      </c>
-      <c r="C4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C8">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 5c3cd46 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/Buch Camille Chronicles/Zeitlinie_Soulbound.xlsx
+++ b/Buch Camille Chronicles/Zeitlinie_Soulbound.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian Dauner\Documents\GitHub\pnpWiki\docs\Buch Camille Chronicles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC6A1844-A1F3-44B1-B0DD-6EFDE1EBED29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6B4AEB4-D3F2-473D-8096-B8FC5BA20C84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="5205" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Monat</t>
   </si>
@@ -43,17 +43,6 @@
   </si>
   <si>
     <t>Asarat</t>
-  </si>
-  <si>
-    <t>Death of Bureaucratess Nalil 
-Camill going to Asarat's Peak
-Camill checks into the bar 'Ubir Ubar’</t>
-  </si>
-  <si>
-    <t>Camill gets thrown from the bar
-Camill attends The Receiving and has a vision from the Immortal Oracle
-Camill gets thrown out of a mercenaries post
-Camill decides to collect moeny for winning in the Arena.</t>
   </si>
   <si>
     <t>Camill fights her first opponent in the Arena
@@ -69,6 +58,29 @@
   </si>
   <si>
     <t>Camill's birthday</t>
+  </si>
+  <si>
+    <t>Camill gets thrown from the bar
+Camill attends The Receiving and has a vision from the Immortal Oracle
+Camill gets thrown out of a mercenaries post
+Camill decides to collect money for winning in the Arena.</t>
+  </si>
+  <si>
+    <t>Camill as a Beggar gets thrown into the Chasm by the Consul, the priest gives her a fake coin as a gift</t>
+  </si>
+  <si>
+    <t>Camill near suicide and joining of Jor's mercenaries</t>
+  </si>
+  <si>
+    <t>Jor explains his plan</t>
+  </si>
+  <si>
+    <t>Festivities of Asarat in the Officiary Palace and Remembrance of Nalli</t>
+  </si>
+  <si>
+    <t>Death of Bureaucratess Nalli 
+Camill going to Asarat's Peak
+Camill checks into the bar 'Ubir Ubar’</t>
   </si>
 </sst>
 </file>
@@ -397,7 +409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="26.109375" bestFit="1" customWidth="1"/>
@@ -406,7 +418,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -426,13 +438,13 @@
         <v>3739</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C2">
         <v>3</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -446,7 +458,7 @@
         <v>52</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="144" x14ac:dyDescent="0.3">
@@ -458,7 +470,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
@@ -466,12 +478,44 @@
         <v>2</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="C8">
         <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="C9">
+        <v>18</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C10">
+        <v>19</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C11">
+        <v>20</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="C15">
+        <v>38</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>